<commit_message>
fix dashboard compact duration labels
</commit_message>
<xml_diff>
--- a/tools/language/多语言对照表.xlsx
+++ b/tools/language/多语言对照表.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="common" sheetId="1" r:id="Rc5fb3d18fecb4eae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="app" sheetId="2" r:id="R427faccaff2145a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="baby_recyclerview" sheetId="3" r:id="R45ae57d448ee4ab2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="common" sheetId="1" r:id="Rf1fd52605813477b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="app" sheetId="2" r:id="Raad3613902024864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="baby_recyclerview" sheetId="3" r:id="Rd47692228b6e4dce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21654,7 +21654,7 @@
         <x:v>%1$d小时%2$d分</x:v>
       </x:c>
       <x:c r="C507" t="str">
-        <x:v>%1$dh %2$dm</x:v>
+        <x:v>%1$dH %2$dm</x:v>
       </x:c>
       <x:c r="D507" t="str">
         <x:v>%1$d小時%2$d分</x:v>
@@ -21696,7 +21696,7 @@
         <x:v>%1$d小时</x:v>
       </x:c>
       <x:c r="C508" t="str">
-        <x:v>%1$dh</x:v>
+        <x:v>%1$dH</x:v>
       </x:c>
       <x:c r="D508" t="str">
         <x:v>%1$d小時</x:v>
@@ -21735,13 +21735,13 @@
         <x:v>summary_duration_minutes_compact</x:v>
       </x:c>
       <x:c r="B509" t="str">
-        <x:v>%1$d分钟</x:v>
+        <x:v>%1$d分</x:v>
       </x:c>
       <x:c r="C509" t="str">
         <x:v>%1$dm</x:v>
       </x:c>
       <x:c r="D509" t="str">
-        <x:v>%1$d分鐘</x:v>
+        <x:v>%1$d分</x:v>
       </x:c>
       <x:c r="E509" t="str">
         <x:v>%1$d分</x:v>
@@ -21777,13 +21777,13 @@
         <x:v>summary_duration_zero_compact</x:v>
       </x:c>
       <x:c r="B510" t="str">
-        <x:v>0分钟</x:v>
+        <x:v>0分</x:v>
       </x:c>
       <x:c r="C510" t="str">
         <x:v>0m</x:v>
       </x:c>
       <x:c r="D510" t="str">
-        <x:v>0分鐘</x:v>
+        <x:v>0分</x:v>
       </x:c>
       <x:c r="E510" t="str">
         <x:v>0分</x:v>
@@ -22363,7 +22363,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12dd8bffd1cc41cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R270e3dc2e53f4d95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22533,7 +22533,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7a26ef3056846c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c4e0e6384c94c86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22829,7 +22829,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb69fdc5f3b69435f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fe23672f9f8443e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>